<commit_message>
feat: implement pauta-excel utility for generating school report spreadsheets and add associated service logic
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
   <si>
     <t>INSTITUTO TÉCNICO PRIVADO DE SAÚDE JOMORAIS</t>
   </si>
@@ -41,10 +41,27 @@
     </r>
   </si>
   <si>
-    <t>11ª CLASSE</t>
-  </si>
-  <si>
-    <t>CURSO: ANÁLISES CLÍNICAS</t>
+    <t>10ª CLASSE</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="26"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">CURSO: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF0070C0"/>
+        <sz val="26"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t/>
+    </r>
   </si>
   <si>
     <r>
@@ -99,24 +116,13 @@
     <t>20/06/26</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF0070C0"/>
-        <sz val="14"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">TURMA: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFFF0000"/>
-        <sz val="14"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>A</t>
-    </r>
+    <t>____________________________</t>
+  </si>
+  <si>
+    <t>TURMA:</t>
+  </si>
+  <si>
+    <t>10ª ÚNICA-ANÁLISES CLÌNICAS-MATINAL</t>
   </si>
   <si>
     <t>M:</t>
@@ -260,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -286,13 +292,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF0070C0"/>
-      <sz val="26"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF333333"/>
+      <color rgb="FF000000"/>
       <sz val="12"/>
       <name val="Blackadder ITC"/>
     </font>
@@ -304,8 +304,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF333333"/>
-      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -316,7 +316,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF555555"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
       <name val="Agency FB"/>
     </font>
@@ -480,7 +480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -493,46 +493,52 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -543,52 +549,49 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1261,14 +1264,14 @@
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
-      <c r="K9" s="6" t="s">
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="P9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
       <c r="R9" s="6"/>
       <c r="S9" s="6"/>
@@ -1300,11 +1303,11 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
@@ -1330,32 +1333,34 @@
       <c r="AK10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="AL10" s="5">
+      <c r="AL10" s="10">
         <f>COUNTIF(R17:R19,"M")+COUNTIF(R17:R19,"F")</f>
       </c>
-      <c r="AM10" s="10" t="s">
+      <c r="AM10" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="AN10" s="10"/>
-      <c r="AO10" s="10"/>
-      <c r="AP10" s="10"/>
+      <c r="AN10" s="11"/>
+      <c r="AO10" s="11"/>
+      <c r="AP10" s="11"/>
     </row>
     <row r="11" ht="20.25" customHeight="1" spans="2:42" x14ac:dyDescent="0.25">
-      <c r="B11" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="G11" s="4" t="s">
+      <c r="B11" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="G11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
       <c r="R11" s="6"/>
@@ -1377,30 +1382,30 @@
       <c r="AI11" s="7"/>
       <c r="AJ11" s="7"/>
       <c r="AK11" s="9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AL11" s="9">
         <f>COUNTIF(R17:R19,"M")</f>
       </c>
-      <c r="AM11" s="10"/>
-      <c r="AN11" s="10"/>
-      <c r="AO11" s="10"/>
-      <c r="AP11" s="10"/>
+      <c r="AM11" s="11"/>
+      <c r="AN11" s="11"/>
+      <c r="AO11" s="11"/>
+      <c r="AP11" s="11"/>
     </row>
     <row r="12" ht="19.5" customHeight="1" spans="2:42" x14ac:dyDescent="0.25">
-      <c r="B12" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
+      <c r="B12" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
       <c r="R12" s="6"/>
@@ -1418,434 +1423,435 @@
       <c r="AD12" s="6"/>
       <c r="AE12" s="6"/>
       <c r="AF12" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AG12" s="7"/>
       <c r="AH12" s="7"/>
       <c r="AI12" s="7"/>
       <c r="AJ12" s="7"/>
       <c r="AK12" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL12" s="14">
+        <f>COUNTIF(R17:R19,"F")</f>
+      </c>
+      <c r="AM12" s="11"/>
+      <c r="AN12" s="11"/>
+      <c r="AO12" s="11"/>
+      <c r="AP12" s="11"/>
+    </row>
+    <row r="13" ht="20.25" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" ht="25" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B14" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q14" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="R14" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="S14" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="T14" s="20"/>
+      <c r="U14" s="20"/>
+      <c r="V14" s="20"/>
+      <c r="W14" s="20"/>
+      <c r="X14" s="20"/>
+      <c r="Y14" s="20"/>
+      <c r="Z14" s="20"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="21"/>
+      <c r="H15" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="21"/>
+      <c r="K15" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="L15" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="M15" s="21"/>
+      <c r="N15" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="19"/>
+      <c r="S15" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="T15" s="21"/>
+      <c r="U15" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="V15" s="21"/>
+      <c r="W15" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="X15" s="21"/>
+      <c r="Y15" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z15" s="21"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="K16" s="22"/>
+      <c r="L16" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="M16" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16" s="22"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="T16" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="U16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="V16" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="W16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="X16" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z16" s="21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B17" s="24">
+        <v>1</v>
+      </c>
+      <c r="C17" s="24">
+        <v>101</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="28">
+        <v>9</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" s="24">
+        <v>2</v>
+      </c>
+      <c r="K17" s="29">
+        <v>14.5</v>
+      </c>
+      <c r="L17" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="M17" s="24">
+        <v>1</v>
+      </c>
+      <c r="N17" s="29">
+        <v>12</v>
+      </c>
+      <c r="O17" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="P17" s="29">
+        <f>AVERAGE(H17,K17,N17)</f>
+      </c>
+      <c r="Q17" s="24">
+        <v>18</v>
+      </c>
+      <c r="R17" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="S17" s="31">
+        <f>COUNTIF(R17:R19,"M")</f>
+      </c>
+      <c r="T17" s="32">
+        <f>COUNTIF(R17:R19,"F")</f>
+      </c>
+      <c r="U17" s="31">
+        <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
+      </c>
+      <c r="V17" s="32">
+        <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
+      </c>
+      <c r="W17" s="31">
+        <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
+      </c>
+      <c r="X17" s="32">
+        <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
+      </c>
+      <c r="Y17" s="31">
+        <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
+      </c>
+      <c r="Z17" s="32">
+        <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B18" s="24">
+        <v>2</v>
+      </c>
+      <c r="C18" s="24">
+        <v>102</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" s="24">
+        <v>1</v>
+      </c>
+      <c r="H18" s="29">
+        <v>11.5</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="J18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="K18" s="29">
+        <v>16</v>
+      </c>
+      <c r="L18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="M18" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="N18" s="29">
         <v>15</v>
       </c>
-      <c r="AL12" s="13">
-        <f>COUNTIF(R17:R19,"F")</f>
-      </c>
-      <c r="AM12" s="10"/>
-      <c r="AN12" s="10"/>
-      <c r="AO12" s="10"/>
-      <c r="AP12" s="10"/>
-    </row>
-    <row r="13" ht="20.25" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-    </row>
-    <row r="14" ht="25" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B14" s="15" t="s">
+      <c r="O18" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="P18" s="29">
+        <f>AVERAGE(H18,K18,N18)</f>
+      </c>
+      <c r="Q18" s="24">
+        <v>19</v>
+      </c>
+      <c r="R18" s="24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B19" s="24">
+        <v>3</v>
+      </c>
+      <c r="C19" s="24">
+        <v>103</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="I19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="J19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="K19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="L19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="M19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="N19" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="O19" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="P19" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q19" s="24">
         <v>17</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="P14" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q14" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R14" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="S14" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="T14" s="19"/>
-      <c r="U14" s="19"/>
-      <c r="V14" s="19"/>
-      <c r="W14" s="19"/>
-      <c r="X14" s="19"/>
-      <c r="Y14" s="19"/>
-      <c r="Z14" s="19"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" s="20"/>
-      <c r="H15" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="I15" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J15" s="20"/>
-      <c r="K15" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="L15" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="M15" s="20"/>
-      <c r="N15" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="O15" s="17"/>
-      <c r="P15" s="17"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="18"/>
-      <c r="S15" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="T15" s="20"/>
-      <c r="U15" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="V15" s="20"/>
-      <c r="W15" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="X15" s="20"/>
-      <c r="Y15" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z15" s="20"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="21"/>
-      <c r="I16" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="J16" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="K16" s="21"/>
-      <c r="L16" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="M16" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="N16" s="21"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="T16" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="U16" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="V16" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="W16" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="X16" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y16" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z16" s="20" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="23">
-        <v>1</v>
-      </c>
-      <c r="C17" s="23">
-        <v>101</v>
-      </c>
-      <c r="D17" s="24" t="s">
+      <c r="R19" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="G17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="H17" s="27">
-        <v>9</v>
-      </c>
-      <c r="I17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="J17" s="23">
-        <v>2</v>
-      </c>
-      <c r="K17" s="28">
-        <v>14.5</v>
-      </c>
-      <c r="L17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="M17" s="23">
-        <v>1</v>
-      </c>
-      <c r="N17" s="28">
-        <v>12</v>
-      </c>
-      <c r="O17" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="P17" s="28">
-        <f>AVERAGE(H17,K17,N17)</f>
-      </c>
-      <c r="Q17" s="23">
-        <v>18</v>
-      </c>
-      <c r="R17" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="S17" s="30">
-        <f>COUNTIF(R17:R19,"M")</f>
-      </c>
-      <c r="T17" s="31">
-        <f>COUNTIF(R17:R19,"F")</f>
-      </c>
-      <c r="U17" s="30">
-        <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
-      </c>
-      <c r="V17" s="31">
-        <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
-      </c>
-      <c r="W17" s="30">
-        <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
-      </c>
-      <c r="X17" s="31">
-        <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
-      </c>
-      <c r="Y17" s="30">
-        <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
-      </c>
-      <c r="Z17" s="31">
-        <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="23">
-        <v>2</v>
-      </c>
-      <c r="C18" s="23">
-        <v>102</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="F18" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="G18" s="23">
-        <v>1</v>
-      </c>
-      <c r="H18" s="28">
-        <v>11.5</v>
-      </c>
-      <c r="I18" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="28">
-        <v>16</v>
-      </c>
-      <c r="L18" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="M18" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="N18" s="28">
-        <v>15</v>
-      </c>
-      <c r="O18" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="P18" s="28">
-        <f>AVERAGE(H18,K18,N18)</f>
-      </c>
-      <c r="Q18" s="23">
-        <v>19</v>
-      </c>
-      <c r="R18" s="23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="23">
-        <v>3</v>
-      </c>
-      <c r="C19" s="23">
-        <v>103</v>
-      </c>
-      <c r="D19" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="H19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="I19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="J19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="K19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="L19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="M19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="N19" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="O19" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="P19" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q19" s="23">
-        <v>17</v>
-      </c>
-      <c r="R19" s="23" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
+      <c r="B21" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="L24" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="M24" s="35"/>
-      <c r="N24" s="35"/>
-      <c r="O24" s="35"/>
+      <c r="B24" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="L24" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="L25" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="M25" s="36"/>
-      <c r="N25" s="36"/>
-      <c r="O25" s="36"/>
+      <c r="B25" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="L25" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
+      <c r="O25" s="37"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="L26" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
-      <c r="O26" s="37"/>
+      <c r="B26" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="L26" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
+      <c r="O26" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="45">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
     <mergeCell ref="C8:AP8"/>
-    <mergeCell ref="G9:I10"/>
-    <mergeCell ref="K9:AE12"/>
+    <mergeCell ref="G9:N10"/>
+    <mergeCell ref="P9:AE12"/>
     <mergeCell ref="AG9:AJ9"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="AG10:AJ11"/>
     <mergeCell ref="AM10:AP12"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G11:I12"/>
+    <mergeCell ref="G11:H12"/>
+    <mergeCell ref="I11:N12"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="AF12:AJ12"/>
     <mergeCell ref="B13:D13"/>

</xml_diff>

<commit_message>
feat: add pauta-excel.util.js to generate dynamic school grading report templates using ExcelJS
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -266,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -322,13 +322,19 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <i/>
+      <sz val="9"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FF005080"/>
       <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -480,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -526,20 +532,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -549,25 +555,25 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -579,19 +585,22 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1454,388 +1463,388 @@
       <c r="C14" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17" t="s">
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17" t="s">
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="18" t="s">
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="P14" s="18" t="s">
+      <c r="P14" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="Q14" s="19" t="s">
+      <c r="Q14" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="R14" s="19" t="s">
+      <c r="R14" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="S14" s="20" t="s">
+      <c r="S14" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="T14" s="20"/>
-      <c r="U14" s="20"/>
-      <c r="V14" s="20"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="20"/>
-      <c r="Y14" s="20"/>
-      <c r="Z14" s="20"/>
+      <c r="T14" s="21"/>
+      <c r="U14" s="21"/>
+      <c r="V14" s="21"/>
+      <c r="W14" s="21"/>
+      <c r="X14" s="21"/>
+      <c r="Y14" s="21"/>
+      <c r="Z14" s="21"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="21" t="s">
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="21"/>
-      <c r="H15" s="22" t="s">
+      <c r="G15" s="22"/>
+      <c r="H15" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="I15" s="21" t="s">
+      <c r="I15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="J15" s="21"/>
-      <c r="K15" s="22" t="s">
+      <c r="J15" s="22"/>
+      <c r="K15" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="L15" s="21" t="s">
+      <c r="L15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="M15" s="21"/>
-      <c r="N15" s="22" t="s">
+      <c r="M15" s="22"/>
+      <c r="N15" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="19"/>
-      <c r="S15" s="21" t="s">
+      <c r="O15" s="19"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="20"/>
+      <c r="S15" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="T15" s="21"/>
-      <c r="U15" s="21" t="s">
+      <c r="T15" s="22"/>
+      <c r="U15" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="V15" s="21"/>
-      <c r="W15" s="21" t="s">
+      <c r="V15" s="22"/>
+      <c r="W15" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="X15" s="21"/>
-      <c r="Y15" s="21" t="s">
+      <c r="X15" s="22"/>
+      <c r="Y15" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="Z15" s="21"/>
+      <c r="Z15" s="22"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="23" t="s">
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="22"/>
-      <c r="I16" s="23" t="s">
+      <c r="H16" s="23"/>
+      <c r="I16" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="J16" s="23" t="s">
+      <c r="J16" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="22"/>
-      <c r="L16" s="23" t="s">
+      <c r="K16" s="23"/>
+      <c r="L16" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="M16" s="23" t="s">
+      <c r="M16" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="N16" s="22"/>
-      <c r="O16" s="18"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="21" t="s">
+      <c r="N16" s="23"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="20"/>
+      <c r="R16" s="20"/>
+      <c r="S16" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="T16" s="21" t="s">
+      <c r="T16" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="U16" s="21" t="s">
+      <c r="U16" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="V16" s="21" t="s">
+      <c r="V16" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="W16" s="21" t="s">
+      <c r="W16" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="X16" s="21" t="s">
+      <c r="X16" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="Y16" s="21" t="s">
+      <c r="Y16" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Z16" s="21" t="s">
+      <c r="Z16" s="22" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="24">
+      <c r="B17" s="25">
         <v>1</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="25">
         <v>101</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="D17" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="28">
+      <c r="H17" s="29">
         <v>9</v>
       </c>
-      <c r="I17" s="27" t="s">
+      <c r="I17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J17" s="24">
+      <c r="J17" s="25">
         <v>2</v>
       </c>
-      <c r="K17" s="29">
+      <c r="K17" s="30">
         <v>14.5</v>
       </c>
-      <c r="L17" s="27" t="s">
+      <c r="L17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="24">
+      <c r="M17" s="25">
         <v>1</v>
       </c>
-      <c r="N17" s="29">
+      <c r="N17" s="30">
         <v>12</v>
       </c>
-      <c r="O17" s="30" t="s">
+      <c r="O17" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="29">
+      <c r="P17" s="30">
         <f>AVERAGE(H17,K17,N17)</f>
       </c>
-      <c r="Q17" s="24">
+      <c r="Q17" s="25">
         <v>18</v>
       </c>
-      <c r="R17" s="24" t="s">
+      <c r="R17" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="S17" s="31">
+      <c r="S17" s="32">
         <f>COUNTIF(R17:R19,"M")</f>
       </c>
-      <c r="T17" s="32">
+      <c r="T17" s="33">
         <f>COUNTIF(R17:R19,"F")</f>
       </c>
-      <c r="U17" s="31">
+      <c r="U17" s="32">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="V17" s="32">
+      <c r="V17" s="33">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="W17" s="31">
+      <c r="W17" s="32">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="X17" s="32">
+      <c r="X17" s="33">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="Y17" s="31">
+      <c r="Y17" s="32">
         <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
       </c>
-      <c r="Z17" s="32">
+      <c r="Z17" s="33">
         <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="24">
+      <c r="B18" s="25">
         <v>2</v>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="25">
         <v>102</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="25">
         <v>1</v>
       </c>
-      <c r="H18" s="29">
+      <c r="H18" s="30">
         <v>11.5</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J18" s="27" t="s">
+      <c r="J18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="29">
+      <c r="K18" s="30">
         <v>16</v>
       </c>
-      <c r="L18" s="27" t="s">
+      <c r="L18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="27" t="s">
+      <c r="M18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="N18" s="29">
+      <c r="N18" s="30">
         <v>15</v>
       </c>
-      <c r="O18" s="30" t="s">
+      <c r="O18" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="29">
+      <c r="P18" s="30">
         <f>AVERAGE(H18,K18,N18)</f>
       </c>
-      <c r="Q18" s="24">
+      <c r="Q18" s="25">
         <v>19</v>
       </c>
-      <c r="R18" s="24" t="s">
+      <c r="R18" s="25" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="24">
+      <c r="B19" s="25">
         <v>3</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="25">
         <v>103</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="27" t="s">
+      <c r="H19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="I19" s="27" t="s">
+      <c r="I19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J19" s="27" t="s">
+      <c r="J19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="27" t="s">
+      <c r="K19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="L19" s="27" t="s">
+      <c r="L19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="27" t="s">
+      <c r="M19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="N19" s="27" t="s">
+      <c r="N19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="O19" s="33" t="s">
+      <c r="O19" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="P19" s="34" t="s">
+      <c r="P19" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q19" s="24">
+      <c r="Q19" s="25">
         <v>17</v>
       </c>
-      <c r="R19" s="24" t="s">
+      <c r="R19" s="25" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="L24" s="36" t="s">
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="L24" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
+      <c r="O24" s="37"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="37" t="s">
+      <c r="B25" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="L25" s="37" t="s">
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="L25" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="M25" s="37"/>
-      <c r="N25" s="37"/>
-      <c r="O25" s="37"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
+      <c r="O25" s="38"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="L26" s="38" t="s">
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="L26" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="M26" s="38"/>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
+      <c r="M26" s="39"/>
+      <c r="N26" s="39"/>
+      <c r="O26" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="45">

</xml_diff>

<commit_message>
feat: add utility to generate Excel school grade reports using ExcelJS
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -169,13 +169,13 @@
     <t>DISCIPLINA A REPETIR</t>
   </si>
   <si>
-    <t>FÍSICA</t>
-  </si>
-  <si>
-    <t>MATEMÁTICA</t>
-  </si>
-  <si>
-    <t>QUÍMICA</t>
+    <t>Física</t>
+  </si>
+  <si>
+    <t>Mat.</t>
+  </si>
+  <si>
+    <t>Química</t>
   </si>
   <si>
     <t>OBS</t>
@@ -328,9 +328,9 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF005080"/>
+      <color rgb="FF0070C0"/>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Agency FB"/>
     </font>
     <font>
       <b/>
@@ -344,18 +344,20 @@
     </font>
     <font>
       <b/>
+      <i/>
       <sz val="8"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFC00000"/>
+      <i/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -413,17 +415,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -531,31 +528,31 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1537,46 +1534,46 @@
       <c r="P15" s="19"/>
       <c r="Q15" s="20"/>
       <c r="R15" s="20"/>
-      <c r="S15" s="22" t="s">
+      <c r="S15" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="T15" s="22"/>
-      <c r="U15" s="22" t="s">
+      <c r="T15" s="24"/>
+      <c r="U15" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="V15" s="22"/>
-      <c r="W15" s="22" t="s">
+      <c r="V15" s="24"/>
+      <c r="W15" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="X15" s="22"/>
-      <c r="Y15" s="22" t="s">
+      <c r="X15" s="24"/>
+      <c r="Y15" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="Z15" s="22"/>
+      <c r="Z15" s="24"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
       <c r="D16" s="17"/>
       <c r="E16" s="17"/>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="24" t="s">
+      <c r="G16" s="22" t="s">
         <v>38</v>
       </c>
       <c r="H16" s="23"/>
-      <c r="I16" s="24" t="s">
+      <c r="I16" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="J16" s="24" t="s">
+      <c r="J16" s="22" t="s">
         <v>38</v>
       </c>
       <c r="K16" s="23"/>
-      <c r="L16" s="24" t="s">
+      <c r="L16" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="M16" s="24" t="s">
+      <c r="M16" s="22" t="s">
         <v>38</v>
       </c>
       <c r="N16" s="23"/>
@@ -1584,28 +1581,28 @@
       <c r="P16" s="19"/>
       <c r="Q16" s="20"/>
       <c r="R16" s="20"/>
-      <c r="S16" s="22" t="s">
+      <c r="S16" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="T16" s="22" t="s">
+      <c r="T16" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="U16" s="22" t="s">
+      <c r="U16" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="V16" s="22" t="s">
+      <c r="V16" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="W16" s="22" t="s">
+      <c r="W16" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="X16" s="22" t="s">
+      <c r="X16" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="Y16" s="22" t="s">
+      <c r="Y16" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="Z16" s="22" t="s">
+      <c r="Z16" s="24" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Excel generation utility to export school academic performance records
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
   <si>
     <t>INSTITUTO TÉCNICO PRIVADO DE SAÚDE JOMORAIS</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>DESISTIDO</t>
+  </si>
+  <si>
+    <t>DATA DO CONSELHO DE TURMA______/______/2026</t>
   </si>
   <si>
     <t>DATA DO CONSELHO DE TURMA ______ / ______ / 2026</t>
@@ -483,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -555,6 +558,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -586,6 +590,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1562,21 +1569,21 @@
       <c r="G16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="23"/>
+      <c r="H16" s="25"/>
       <c r="I16" s="22" t="s">
         <v>37</v>
       </c>
       <c r="J16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="23"/>
+      <c r="K16" s="25"/>
       <c r="L16" s="22" t="s">
         <v>37</v>
       </c>
       <c r="M16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="N16" s="23"/>
+      <c r="N16" s="25"/>
       <c r="O16" s="19"/>
       <c r="P16" s="19"/>
       <c r="Q16" s="20"/>
@@ -1607,244 +1614,265 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="25">
+      <c r="B17" s="26">
         <v>1</v>
       </c>
-      <c r="C17" s="25">
+      <c r="C17" s="26">
         <v>101</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="28" t="s">
+      <c r="G17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="29">
+      <c r="H17" s="30">
         <v>9</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="I17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="26">
         <v>2</v>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="31">
         <v>14.5</v>
       </c>
-      <c r="L17" s="28" t="s">
+      <c r="L17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="25">
+      <c r="M17" s="26">
         <v>1</v>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="31">
         <v>12</v>
       </c>
-      <c r="O17" s="31" t="s">
+      <c r="O17" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="31">
         <f>AVERAGE(H17,K17,N17)</f>
       </c>
-      <c r="Q17" s="25">
+      <c r="Q17" s="26">
         <v>18</v>
       </c>
-      <c r="R17" s="25" t="s">
+      <c r="R17" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="S17" s="32">
+      <c r="S17" s="33">
         <f>COUNTIF(R17:R19,"M")</f>
       </c>
-      <c r="T17" s="33">
+      <c r="T17" s="34">
         <f>COUNTIF(R17:R19,"F")</f>
       </c>
-      <c r="U17" s="32">
+      <c r="U17" s="33">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="V17" s="33">
+      <c r="V17" s="34">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="W17" s="32">
+      <c r="W17" s="33">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="X17" s="33">
+      <c r="X17" s="34">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="Y17" s="32">
+      <c r="Y17" s="33">
         <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
       </c>
-      <c r="Z17" s="33">
+      <c r="Z17" s="34">
         <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="25">
+      <c r="B18" s="26">
         <v>2</v>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="26">
         <v>102</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="26">
         <v>1</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="31">
         <v>11.5</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="I18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="J18" s="28" t="s">
+      <c r="J18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="30">
+      <c r="K18" s="31">
         <v>16</v>
       </c>
-      <c r="L18" s="28" t="s">
+      <c r="L18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="28" t="s">
+      <c r="M18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="N18" s="30">
+      <c r="N18" s="31">
         <v>15</v>
       </c>
-      <c r="O18" s="31" t="s">
+      <c r="O18" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="30">
+      <c r="P18" s="31">
         <f>AVERAGE(H18,K18,N18)</f>
       </c>
-      <c r="Q18" s="25">
+      <c r="Q18" s="26">
         <v>19</v>
       </c>
-      <c r="R18" s="25" t="s">
+      <c r="R18" s="26" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="25">
+      <c r="B19" s="26">
         <v>3</v>
       </c>
-      <c r="C19" s="25">
+      <c r="C19" s="26">
         <v>103</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="28" t="s">
+      <c r="G19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="I19" s="28" t="s">
+      <c r="I19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="J19" s="28" t="s">
+      <c r="J19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="28" t="s">
+      <c r="K19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="L19" s="28" t="s">
+      <c r="L19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="28" t="s">
+      <c r="M19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="N19" s="28" t="s">
+      <c r="N19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="O19" s="34" t="s">
+      <c r="O19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="P19" s="35" t="s">
+      <c r="P19" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="Q19" s="25">
+      <c r="Q19" s="26">
         <v>17</v>
       </c>
-      <c r="R19" s="25" t="s">
+      <c r="R19" s="26" t="s">
         <v>39</v>
       </c>
     </row>
+    <row r="20" ht="25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25"/>
+      <c r="M20" s="25"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="25"/>
+      <c r="R20" s="25"/>
+    </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
+      <c r="B21" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="L24" s="37" t="s">
+      <c r="B24" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="M24" s="37"/>
-      <c r="N24" s="37"/>
-      <c r="O24" s="37"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="L24" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="M24" s="39"/>
+      <c r="N24" s="39"/>
+      <c r="O24" s="39"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="L25" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="M25" s="38"/>
-      <c r="N25" s="38"/>
-      <c r="O25" s="38"/>
+      <c r="B25" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="L25" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
+      <c r="O25" s="40"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="39" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="L26" s="39" t="s">
+      <c r="B26" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="M26" s="39"/>
-      <c r="N26" s="39"/>
-      <c r="O26" s="39"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="L26" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="M26" s="41"/>
+      <c r="N26" s="41"/>
+      <c r="O26" s="41"/>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="42">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
@@ -1880,9 +1908,6 @@
     <mergeCell ref="U15:V15"/>
     <mergeCell ref="W15:X15"/>
     <mergeCell ref="Y15:Z15"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="N15:N16"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="L24:O24"/>

</xml_diff>

<commit_message>
feat: implement Excel template generation utility for school grading records
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
   <si>
     <t>INSTITUTO TÉCNICO PRIVADO DE SAÚDE JOMORAIS</t>
   </si>
@@ -239,9 +239,6 @@
   </si>
   <si>
     <t>DESISTIDO</t>
-  </si>
-  <si>
-    <t>DATA DO CONSELHO DE TURMA______/______/2026</t>
   </si>
   <si>
     <t>DATA DO CONSELHO DE TURMA ______ / ______ / 2026</t>
@@ -486,7 +483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -590,9 +587,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1797,12 +1791,12 @@
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="37" t="s">
+      <c r="B20" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="E20" s="25"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="25"/>
       <c r="G20" s="25"/>
       <c r="H20" s="25"/>
@@ -1818,61 +1812,61 @@
       <c r="R20" s="25"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B24" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="39" t="s">
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="L24" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="L24" s="39" t="s">
+      <c r="M24" s="38"/>
+      <c r="N24" s="38"/>
+      <c r="O24" s="38"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="M24" s="39"/>
-      <c r="N24" s="39"/>
-      <c r="O24" s="39"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="40" t="s">
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="L25" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="M25" s="39"/>
+      <c r="N25" s="39"/>
+      <c r="O25" s="39"/>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B26" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="L25" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="M25" s="40"/>
-      <c r="N25" s="40"/>
-      <c r="O25" s="40"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="41" t="s">
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="L26" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="L26" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="M26" s="41"/>
-      <c r="N26" s="41"/>
-      <c r="O26" s="41"/>
+      <c r="M26" s="40"/>
+      <c r="N26" s="40"/>
+      <c r="O26" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
@@ -1908,6 +1902,7 @@
     <mergeCell ref="U15:V15"/>
     <mergeCell ref="W15:X15"/>
     <mergeCell ref="Y15:Z15"/>
+    <mergeCell ref="B20:E20"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="L24:O24"/>

</xml_diff>

<commit_message>
feat: add pauta-excel.util.js to generate school assessment Excel reports using ExcelJS
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
   <si>
     <t>INSTITUTO TÉCNICO PRIVADO DE SAÚDE JOMORAIS</t>
   </si>
@@ -483,7 +483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -588,9 +588,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -984,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:AP26"/>
+  <dimension ref="B1:AP25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1790,7 +1787,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" ht="25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="20" ht="25" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="26" t="s">
         <v>47</v>
       </c>
@@ -1806,30 +1803,32 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25"/>
-      <c r="P20" s="25"/>
-      <c r="Q20" s="25"/>
-      <c r="R20" s="25"/>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="L23" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="37"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B24" s="38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C24" s="38"/>
       <c r="D24" s="38"/>
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
       <c r="L24" s="38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M24" s="38"/>
       <c r="N24" s="38"/>
@@ -1837,36 +1836,21 @@
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B25" s="39" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
       <c r="E25" s="39"/>
       <c r="F25" s="39"/>
       <c r="L25" s="39" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M25" s="39"/>
       <c r="N25" s="39"/>
       <c r="O25" s="39"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
-      <c r="L26" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="M26" s="40"/>
-      <c r="N26" s="40"/>
-      <c r="O26" s="40"/>
-    </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="42">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
@@ -1903,13 +1887,12 @@
     <mergeCell ref="W15:X15"/>
     <mergeCell ref="Y15:Z15"/>
     <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="L23:O23"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="L24:O24"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="L25:O25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="L26:O26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: implement pauta excel template generator utility
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -1850,7 +1850,7 @@
       <c r="O25" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="45">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
@@ -1887,6 +1887,9 @@
     <mergeCell ref="W15:X15"/>
     <mergeCell ref="Y15:Z15"/>
     <mergeCell ref="B20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="L20:M20"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="L23:O23"/>
     <mergeCell ref="B24:F24"/>

</xml_diff>

<commit_message>
feat: implement pauta-excel.util.js to generate school grade reports using ExcelJS
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -266,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -409,6 +409,11 @@
       <color rgb="FF7F7F7F"/>
       <sz val="9"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Blackadder ITC"/>
     </font>
     <font>
       <sz val="11"/>
@@ -555,7 +560,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -589,10 +593,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1560,21 +1565,21 @@
       <c r="G16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="25"/>
+      <c r="H16" s="23"/>
       <c r="I16" s="22" t="s">
         <v>37</v>
       </c>
       <c r="J16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="25"/>
+      <c r="K16" s="23"/>
       <c r="L16" s="22" t="s">
         <v>37</v>
       </c>
       <c r="M16" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="N16" s="25"/>
+      <c r="N16" s="23"/>
       <c r="O16" s="19"/>
       <c r="P16" s="19"/>
       <c r="Q16" s="20"/>
@@ -1605,204 +1610,204 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="26">
+      <c r="B17" s="25">
         <v>1</v>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="25">
         <v>101</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="29" t="s">
+      <c r="F17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="29" t="s">
+      <c r="G17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="29">
         <v>9</v>
       </c>
-      <c r="I17" s="29" t="s">
+      <c r="I17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J17" s="26">
+      <c r="J17" s="25">
         <v>2</v>
       </c>
-      <c r="K17" s="31">
+      <c r="K17" s="30">
         <v>14.5</v>
       </c>
-      <c r="L17" s="29" t="s">
+      <c r="L17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="26">
+      <c r="M17" s="25">
         <v>1</v>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="30">
         <v>12</v>
       </c>
-      <c r="O17" s="32" t="s">
+      <c r="O17" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="30">
         <f>AVERAGE(H17,K17,N17)</f>
       </c>
-      <c r="Q17" s="26">
+      <c r="Q17" s="25">
         <v>18</v>
       </c>
-      <c r="R17" s="26" t="s">
+      <c r="R17" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="S17" s="33">
+      <c r="S17" s="32">
         <f>COUNTIF(R17:R19,"M")</f>
       </c>
-      <c r="T17" s="34">
+      <c r="T17" s="33">
         <f>COUNTIF(R17:R19,"F")</f>
       </c>
-      <c r="U17" s="33">
+      <c r="U17" s="32">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="V17" s="34">
+      <c r="V17" s="33">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="W17" s="33">
+      <c r="W17" s="32">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="X17" s="34">
+      <c r="X17" s="33">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="Y17" s="33">
+      <c r="Y17" s="32">
         <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
       </c>
-      <c r="Z17" s="34">
+      <c r="Z17" s="33">
         <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="26">
+      <c r="B18" s="25">
         <v>2</v>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="25">
         <v>102</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="26">
+      <c r="G18" s="25">
         <v>1</v>
       </c>
-      <c r="H18" s="31">
+      <c r="H18" s="30">
         <v>11.5</v>
       </c>
-      <c r="I18" s="29" t="s">
+      <c r="I18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J18" s="29" t="s">
+      <c r="J18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="31">
+      <c r="K18" s="30">
         <v>16</v>
       </c>
-      <c r="L18" s="29" t="s">
+      <c r="L18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="29" t="s">
+      <c r="M18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="N18" s="31">
+      <c r="N18" s="30">
         <v>15</v>
       </c>
-      <c r="O18" s="32" t="s">
+      <c r="O18" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="31">
+      <c r="P18" s="30">
         <f>AVERAGE(H18,K18,N18)</f>
       </c>
-      <c r="Q18" s="26">
+      <c r="Q18" s="25">
         <v>19</v>
       </c>
-      <c r="R18" s="26" t="s">
+      <c r="R18" s="25" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="26">
+      <c r="B19" s="25">
         <v>3</v>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="25">
         <v>103</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F19" s="29" t="s">
+      <c r="F19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="29" t="s">
+      <c r="H19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="I19" s="29" t="s">
+      <c r="I19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J19" s="29" t="s">
+      <c r="J19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="29" t="s">
+      <c r="K19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="L19" s="29" t="s">
+      <c r="L19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="29" t="s">
+      <c r="M19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="N19" s="29" t="s">
+      <c r="N19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="O19" s="35" t="s">
+      <c r="O19" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="P19" s="36" t="s">
+      <c r="P19" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q19" s="26">
+      <c r="Q19" s="25">
         <v>17</v>
       </c>
-      <c r="R19" s="26" t="s">
+      <c r="R19" s="25" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="25"/>
-      <c r="N20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="36"/>
+      <c r="M20" s="36"/>
+      <c r="N20" s="36"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B23" s="37" t="s">
@@ -1850,7 +1855,7 @@
       <c r="O25" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="48">
     <mergeCell ref="D2:AP4"/>
     <mergeCell ref="B5:AP5"/>
     <mergeCell ref="B7:AP7"/>
@@ -1886,6 +1891,9 @@
     <mergeCell ref="U15:V15"/>
     <mergeCell ref="W15:X15"/>
     <mergeCell ref="Y15:Z15"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="N15:N16"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="I20:J20"/>

</xml_diff>

<commit_message>
feat: implement pauta-excel.util.js to generate Excel reports and add utility script for font styling adjustments
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -266,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -362,34 +362,34 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <i/>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <color rgb="FF7F7F7F"/>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFF0000"/>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0070C0"/>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="Arial Narrow"/>
     </font>
     <font>
       <b/>
@@ -407,6 +407,10 @@
       <b/>
       <i/>
       <color rgb="FF7F7F7F"/>
+      <sz val="9"/>
+      <name val="Arial Narrow"/>
+    </font>
+    <font>
       <sz val="9"/>
       <name val="Calibri"/>
     </font>
@@ -488,7 +492,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -593,11 +597,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1793,66 +1800,66 @@
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="36"/>
-      <c r="K20" s="36"/>
-      <c r="L20" s="36"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="37"/>
+      <c r="M20" s="37"/>
+      <c r="N20" s="37"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="37" t="s">
+      <c r="B23" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="L23" s="37" t="s">
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="L23" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="M23" s="37"/>
-      <c r="N23" s="37"/>
-      <c r="O23" s="37"/>
+      <c r="M23" s="38"/>
+      <c r="N23" s="38"/>
+      <c r="O23" s="38"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="L24" s="38" t="s">
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="L24" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="M24" s="38"/>
-      <c r="N24" s="38"/>
-      <c r="O24" s="38"/>
+      <c r="M24" s="39"/>
+      <c r="N24" s="39"/>
+      <c r="O24" s="39"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="L25" s="39" t="s">
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="L25" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="M25" s="39"/>
-      <c r="N25" s="39"/>
-      <c r="O25" s="39"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
+      <c r="O25" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="48">

</xml_diff>

<commit_message>
feat: implement Pauta Excel template generator using exceljs
</commit_message>
<xml_diff>
--- a/jomorais-backend/scratch/test_output.xlsx
+++ b/jomorais-backend/scratch/test_output.xlsx
@@ -323,7 +323,7 @@
     <font>
       <b/>
       <i/>
-      <sz val="9"/>
+      <sz val="14"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -361,17 +361,16 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Arial Narrow"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Arial Narrow"/>
     </font>
     <font>
-      <i/>
-      <sz val="8"/>
+      <sz val="11"/>
       <name val="Arial Narrow"/>
     </font>
     <font>
@@ -492,7 +491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -543,6 +542,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -568,6 +570,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1473,393 +1478,393 @@
       <c r="D14" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18" t="s">
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18" t="s">
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="19" t="s">
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="P14" s="19" t="s">
+      <c r="P14" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="Q14" s="20" t="s">
+      <c r="Q14" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="R14" s="20" t="s">
+      <c r="R14" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="S14" s="21" t="s">
+      <c r="S14" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="T14" s="21"/>
-      <c r="U14" s="21"/>
-      <c r="V14" s="21"/>
-      <c r="W14" s="21"/>
-      <c r="X14" s="21"/>
-      <c r="Y14" s="21"/>
-      <c r="Z14" s="21"/>
+      <c r="T14" s="22"/>
+      <c r="U14" s="22"/>
+      <c r="V14" s="22"/>
+      <c r="W14" s="22"/>
+      <c r="X14" s="22"/>
+      <c r="Y14" s="22"/>
+      <c r="Z14" s="22"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="22" t="s">
+      <c r="E15" s="18"/>
+      <c r="F15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23" t="s">
+      <c r="G15" s="23"/>
+      <c r="H15" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="I15" s="22" t="s">
+      <c r="I15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="J15" s="22"/>
-      <c r="K15" s="23" t="s">
+      <c r="J15" s="23"/>
+      <c r="K15" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="L15" s="22" t="s">
+      <c r="L15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="M15" s="22"/>
-      <c r="N15" s="23" t="s">
+      <c r="M15" s="23"/>
+      <c r="N15" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="O15" s="19"/>
-      <c r="P15" s="19"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="24" t="s">
+      <c r="O15" s="20"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
+      <c r="S15" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="T15" s="24"/>
-      <c r="U15" s="24" t="s">
+      <c r="T15" s="25"/>
+      <c r="U15" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="V15" s="24"/>
-      <c r="W15" s="24" t="s">
+      <c r="V15" s="25"/>
+      <c r="W15" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="X15" s="24"/>
-      <c r="Y15" s="24" t="s">
+      <c r="X15" s="25"/>
+      <c r="Y15" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="Z15" s="24"/>
+      <c r="Z15" s="25"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="22" t="s">
+      <c r="E16" s="18"/>
+      <c r="F16" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="23"/>
-      <c r="I16" s="22" t="s">
+      <c r="H16" s="24"/>
+      <c r="I16" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="J16" s="22" t="s">
+      <c r="J16" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="23"/>
-      <c r="L16" s="22" t="s">
+      <c r="K16" s="24"/>
+      <c r="L16" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="N16" s="23"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="19"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="24" t="s">
+      <c r="N16" s="24"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="21"/>
+      <c r="R16" s="21"/>
+      <c r="S16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="T16" s="24" t="s">
+      <c r="T16" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="U16" s="24" t="s">
+      <c r="U16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="V16" s="24" t="s">
+      <c r="V16" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="W16" s="24" t="s">
+      <c r="W16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="X16" s="24" t="s">
+      <c r="X16" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="Y16" s="24" t="s">
+      <c r="Y16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="Z16" s="24" t="s">
+      <c r="Z16" s="25" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="25">
+      <c r="B17" s="26">
         <v>1</v>
       </c>
-      <c r="C17" s="25">
+      <c r="C17" s="27">
         <v>101</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="28" t="s">
+      <c r="G17" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="29">
+      <c r="H17" s="31">
         <v>9</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="I17" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="27">
         <v>2</v>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="32">
         <v>14.5</v>
       </c>
-      <c r="L17" s="28" t="s">
+      <c r="L17" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="25">
+      <c r="M17" s="27">
         <v>1</v>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="32">
         <v>12</v>
       </c>
-      <c r="O17" s="31" t="s">
+      <c r="O17" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="32">
         <f>AVERAGE(H17,K17,N17)</f>
       </c>
-      <c r="Q17" s="25">
+      <c r="Q17" s="27">
         <v>18</v>
       </c>
-      <c r="R17" s="25" t="s">
+      <c r="R17" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="S17" s="32">
+      <c r="S17" s="34">
         <f>COUNTIF(R17:R19,"M")</f>
       </c>
-      <c r="T17" s="33">
+      <c r="T17" s="35">
         <f>COUNTIF(R17:R19,"F")</f>
       </c>
-      <c r="U17" s="32">
+      <c r="U17" s="34">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="V17" s="33">
+      <c r="V17" s="35">
         <f>COUNTIFS(O17:O19,"TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="W17" s="32">
+      <c r="W17" s="34">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"M")</f>
       </c>
-      <c r="X17" s="33">
+      <c r="X17" s="35">
         <f>COUNTIFS(O17:O19,"N/TRANSITA",R17:R19,"F")</f>
       </c>
-      <c r="Y17" s="32">
+      <c r="Y17" s="34">
         <f>COUNTIFS(O17:O19,"DESISTIDO",R17:R19,"M")</f>
       </c>
-      <c r="Z17" s="33">
+      <c r="Z17" s="35">
         <f>COUNTIFS(O17:O19,"DESISTIDA",R17:R19,"F")</f>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="25">
+      <c r="B18" s="26">
         <v>2</v>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="27">
         <v>102</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="27">
         <v>1</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="32">
         <v>11.5</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="I18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="J18" s="28" t="s">
+      <c r="J18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="30">
+      <c r="K18" s="32">
         <v>16</v>
       </c>
-      <c r="L18" s="28" t="s">
+      <c r="L18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="28" t="s">
+      <c r="M18" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N18" s="30">
+      <c r="N18" s="32">
         <v>15</v>
       </c>
-      <c r="O18" s="31" t="s">
+      <c r="O18" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="P18" s="30">
+      <c r="P18" s="32">
         <f>AVERAGE(H18,K18,N18)</f>
       </c>
-      <c r="Q18" s="25">
+      <c r="Q18" s="27">
         <v>19</v>
       </c>
-      <c r="R18" s="25" t="s">
+      <c r="R18" s="27" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="25">
+      <c r="B19" s="26">
         <v>3</v>
       </c>
-      <c r="C19" s="25">
+      <c r="C19" s="27">
         <v>103</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="28" t="s">
+      <c r="G19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="I19" s="28" t="s">
+      <c r="I19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="J19" s="28" t="s">
+      <c r="J19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="28" t="s">
+      <c r="K19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="L19" s="28" t="s">
+      <c r="L19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="28" t="s">
+      <c r="M19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N19" s="28" t="s">
+      <c r="N19" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="O19" s="34" t="s">
+      <c r="O19" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="P19" s="35" t="s">
+      <c r="P19" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="Q19" s="25">
+      <c r="Q19" s="27">
         <v>17</v>
       </c>
-      <c r="R19" s="25" t="s">
+      <c r="R19" s="27" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="37"/>
-      <c r="K20" s="37"/>
-      <c r="L20" s="37"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="37"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
+      <c r="L20" s="39"/>
+      <c r="M20" s="39"/>
+      <c r="N20" s="39"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="38" t="s">
+      <c r="B23" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
-      <c r="L23" s="38" t="s">
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="L23" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="M23" s="38"/>
-      <c r="N23" s="38"/>
-      <c r="O23" s="38"/>
+      <c r="M23" s="40"/>
+      <c r="N23" s="40"/>
+      <c r="O23" s="40"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="39" t="s">
+      <c r="B24" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="L24" s="39" t="s">
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="L24" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="M24" s="39"/>
-      <c r="N24" s="39"/>
-      <c r="O24" s="39"/>
+      <c r="M24" s="41"/>
+      <c r="N24" s="41"/>
+      <c r="O24" s="41"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="L25" s="40" t="s">
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="L25" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="M25" s="40"/>
-      <c r="N25" s="40"/>
-      <c r="O25" s="40"/>
+      <c r="M25" s="42"/>
+      <c r="N25" s="42"/>
+      <c r="O25" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="48">

</xml_diff>